<commit_message>
auto sync 2026-07-08 11:25:11
</commit_message>
<xml_diff>
--- a/BOM_zero_case.xlsx
+++ b/BOM_zero_case.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="56">
   <si>
     <t>No.</t>
   </si>
@@ -167,10 +167,10 @@
     <t>M3*6</t>
   </si>
   <si>
-    <t>M2.5*7</t>
-  </si>
-  <si>
-    <t>M2.5*15</t>
+    <t>M2.5*8</t>
+  </si>
+  <si>
+    <t>M2.5*14</t>
   </si>
   <si>
     <t>M2.5</t>
@@ -179,6 +179,12 @@
     <t>尼龙螺母</t>
   </si>
   <si>
+    <t>4*2.7*2</t>
+  </si>
+  <si>
+    <t>隔离柱</t>
+  </si>
+  <si>
     <t>320*172 262k</t>
   </si>
   <si>
@@ -186,6 +192,9 @@
   </si>
   <si>
     <t>ST7789 TFT彩屏</t>
+  </si>
+  <si>
+    <t>亚克力板 硅橡胶 焊锡</t>
   </si>
 </sst>
 </file>
@@ -1193,7 +1202,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="5.36363636363636" customWidth="1"/>
@@ -1526,14 +1535,14 @@
       <c r="A18" s="2">
         <v>17</v>
       </c>
-      <c r="B18" s="3">
+      <c r="B18" s="2">
         <v>4</v>
       </c>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3" t="s">
+      <c r="C18" s="2"/>
+      <c r="D18" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="E18" s="2" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1557,16 +1566,39 @@
         <v>19</v>
       </c>
       <c r="B20" s="2">
+        <v>4</v>
+      </c>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" s="3">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2">
         <v>1</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E20" s="2" t="s">
+      <c r="C21" s="2" t="s">
         <v>52</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" s="3">
+        <v>21</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto sync 2026-07-08 11:25:31
</commit_message>
<xml_diff>
--- a/BOM_zero_case.xlsx
+++ b/BOM_zero_case.xlsx
@@ -808,13 +808,10 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1577,7 +1574,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="3">
+      <c r="A21" s="2">
         <v>20</v>
       </c>
       <c r="B21" s="2">
@@ -1594,10 +1591,8 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="3">
-        <v>21</v>
-      </c>
-      <c r="E22" s="3" t="s">
+      <c r="A22" s="2"/>
+      <c r="E22" s="2" t="s">
         <v>55</v>
       </c>
     </row>

</xml_diff>

<commit_message>
auto sync 2026-07-12 23:10:43
</commit_message>
<xml_diff>
--- a/BOM_zero_case.xlsx
+++ b/BOM_zero_case.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="59">
   <si>
     <t>No.</t>
   </si>
@@ -194,7 +194,16 @@
     <t>ST7789 TFT彩屏</t>
   </si>
   <si>
-    <t>亚克力板 硅橡胶 焊锡</t>
+    <t>84*27*1mm</t>
+  </si>
+  <si>
+    <t>亚克力板</t>
+  </si>
+  <si>
+    <t>84*28*1mm</t>
+  </si>
+  <si>
+    <t>硅橡胶 焊锡</t>
   </si>
 </sst>
 </file>
@@ -808,13 +817,16 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1199,7 +1211,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="5.36363636363636" customWidth="1"/>
@@ -1513,7 +1525,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:6">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -1528,7 +1540,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:6">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -1543,7 +1555,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:6">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -1558,7 +1570,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:6">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -1573,7 +1585,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:6">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -1590,11 +1602,49 @@
         <v>54</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
-      <c r="A22" s="2"/>
-      <c r="E22" s="2" t="s">
+    <row r="22" spans="1:6">
+      <c r="A22" s="1">
+        <v>21</v>
+      </c>
+      <c r="B22" s="3">
+        <v>1</v>
+      </c>
+      <c r="C22" s="3" t="s">
         <v>55</v>
       </c>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F22" s="3"/>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" s="3">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3">
+        <v>1</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F23" s="3"/>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" s="3">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F24" s="3"/>
     </row>
   </sheetData>
   <printOptions gridLines="1"/>

</xml_diff>